<commit_message>
Fix domain and nature columns in systems Excel export
The source classifier puts every executive bylaw (اللائحة التنفيذية) under the
enforcement domain because of the word itself; bylaws now inherit their
parent system's domain and nature. Procedural/judicial nature uses name
rules so courts, judicial costs and Board of Grievances systems are no
longer marked substantive. Parent system is filled for bylaws, and names
are kept exactly as in the source.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K9EdjfPD5SRmJTSSVgGr8W
</commit_message>
<xml_diff>
--- a/reports/saudi-systems-issuance.xlsx
+++ b/reports/saudi-systems-issuance.xlsx
@@ -14,7 +14,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'الأنظمة'!$A$1:$M$501</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'المؤرخة'!$A$1:$H$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ملخص'!$A$1:$B$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ملخص'!$A$1:$B$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -785,7 +785,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>موضوعي/تنظيمي</t>
+          <t>قضائي تنظيمي</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr"/>
@@ -1086,7 +1086,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>التنفيذ</t>
+          <t>المرافعات والإجراءات</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -1094,7 +1094,11 @@
           <t>إجرائي</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr"/>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>نظام الإجراءات الجزائية</t>
+        </is>
+      </c>
       <c r="H12" s="5" t="n">
         <v>181</v>
       </c>
@@ -1528,15 +1532,19 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>التنفيذ</t>
+          <t>الشركات</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>إجرائي</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="inlineStr"/>
+          <t>موضوعي/تنظيمي</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>نظام الإفلاس</t>
+        </is>
+      </c>
       <c r="H22" s="5" t="n">
         <v>98</v>
       </c>
@@ -1576,7 +1584,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>موضوعي/تنظيمي</t>
+          <t>إجرائي</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
@@ -1803,7 +1811,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>موضوعي/تنظيمي</t>
+          <t>قضائي تنظيمي</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr"/>
@@ -2354,7 +2362,7 @@
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>أخرى</t>
+          <t>نظام</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -3931,15 +3939,19 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t>التنفيذ</t>
+          <t>الجزائي والعقوبات</t>
         </is>
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>إجرائي</t>
-        </is>
-      </c>
-      <c r="G77" s="5" t="inlineStr"/>
+          <t>موضوعي/تنظيمي</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>نظام مكافحة المخدرات والمؤثرات العقلية</t>
+        </is>
+      </c>
       <c r="H77" s="5" t="n">
         <v>40</v>
       </c>
@@ -6000,7 +6012,7 @@
       </c>
       <c r="F125" s="5" t="inlineStr">
         <is>
-          <t>موضوعي/تنظيمي</t>
+          <t>قضائي تنظيمي</t>
         </is>
       </c>
       <c r="G125" s="5" t="inlineStr"/>
@@ -6043,7 +6055,7 @@
       </c>
       <c r="F126" s="5" t="inlineStr">
         <is>
-          <t>موضوعي/تنظيمي</t>
+          <t>قضائي تنظيمي</t>
         </is>
       </c>
       <c r="G126" s="5" t="inlineStr"/>
@@ -7070,15 +7082,19 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t>التنفيذ</t>
+          <t>الجزائي والعقوبات</t>
         </is>
       </c>
       <c r="F150" s="5" t="inlineStr">
         <is>
-          <t>إجرائي</t>
-        </is>
-      </c>
-      <c r="G150" s="5" t="inlineStr"/>
+          <t>موضوعي/تنظيمي</t>
+        </is>
+      </c>
+      <c r="G150" s="5" t="inlineStr">
+        <is>
+          <t>نظام مكافحة جرائم الإرهاب وتمويله</t>
+        </is>
+      </c>
       <c r="H150" s="5" t="n">
         <v>26</v>
       </c>
@@ -7156,15 +7172,19 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t>التنفيذ</t>
+          <t>العقار والتسجيل العيني</t>
         </is>
       </c>
       <c r="F152" s="5" t="inlineStr">
         <is>
-          <t>إجرائي</t>
-        </is>
-      </c>
-      <c r="G152" s="5" t="inlineStr"/>
+          <t>موضوعي/تنظيمي</t>
+        </is>
+      </c>
+      <c r="G152" s="5" t="inlineStr">
+        <is>
+          <t>نظام نزع ملكية العقارات للمنفعة العامة ووضع اليد المؤقت على العقار</t>
+        </is>
+      </c>
       <c r="H152" s="5" t="n">
         <v>26</v>
       </c>
@@ -7247,7 +7267,7 @@
       </c>
       <c r="F154" s="5" t="inlineStr">
         <is>
-          <t>موضوعي/تنظيمي</t>
+          <t>قضائي تنظيمي</t>
         </is>
       </c>
       <c r="G154" s="5" t="inlineStr"/>
@@ -7973,12 +7993,12 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t>التنفيذ</t>
+          <t>غير مصنف</t>
         </is>
       </c>
       <c r="F171" s="5" t="inlineStr">
         <is>
-          <t>إجرائي</t>
+          <t>موضوعي/تنظيمي</t>
         </is>
       </c>
       <c r="G171" s="5" t="inlineStr"/>
@@ -8322,7 +8342,7 @@
       </c>
       <c r="F179" s="5" t="inlineStr">
         <is>
-          <t>موضوعي/تنظيمي</t>
+          <t>إجرائي</t>
         </is>
       </c>
       <c r="G179" s="5" t="inlineStr"/>
@@ -10133,7 +10153,11 @@
           <t>إجرائي</t>
         </is>
       </c>
-      <c r="G221" s="5" t="inlineStr"/>
+      <c r="G221" s="5" t="inlineStr">
+        <is>
+          <t>نظام التحكيم</t>
+        </is>
+      </c>
       <c r="H221" s="5" t="n">
         <v>19</v>
       </c>
@@ -10942,15 +10966,19 @@
       </c>
       <c r="E240" s="5" t="inlineStr">
         <is>
-          <t>التنفيذ</t>
+          <t>تنظيمي قطاعي</t>
         </is>
       </c>
       <c r="F240" s="5" t="inlineStr">
         <is>
-          <t>إجرائي</t>
-        </is>
-      </c>
-      <c r="G240" s="5" t="inlineStr"/>
+          <t>موضوعي/تنظيمي</t>
+        </is>
+      </c>
+      <c r="G240" s="5" t="inlineStr">
+        <is>
+          <t>نظام رسوم الأراضي البيضاء</t>
+        </is>
+      </c>
       <c r="H240" s="5" t="n">
         <v>18</v>
       </c>
@@ -11976,7 +12004,7 @@
       </c>
       <c r="E264" s="5" t="inlineStr">
         <is>
-          <t>التنفيذ</t>
+          <t>تنظيمي قطاعي</t>
         </is>
       </c>
       <c r="F264" s="5" t="inlineStr">
@@ -11984,7 +12012,11 @@
           <t>إجرائي</t>
         </is>
       </c>
-      <c r="G264" s="5" t="inlineStr"/>
+      <c r="G264" s="5" t="inlineStr">
+        <is>
+          <t>نظام التكاليف القضائية</t>
+        </is>
+      </c>
       <c r="H264" s="5" t="n">
         <v>17</v>
       </c>
@@ -13223,15 +13255,19 @@
       </c>
       <c r="E293" s="5" t="inlineStr">
         <is>
-          <t>التنفيذ</t>
+          <t>تنظيمي قطاعي</t>
         </is>
       </c>
       <c r="F293" s="5" t="inlineStr">
         <is>
-          <t>إجرائي</t>
-        </is>
-      </c>
-      <c r="G293" s="5" t="inlineStr"/>
+          <t>موضوعي/تنظيمي</t>
+        </is>
+      </c>
+      <c r="G293" s="5" t="inlineStr">
+        <is>
+          <t>نظام الأوسمة السعودية</t>
+        </is>
+      </c>
       <c r="H293" s="5" t="n">
         <v>16</v>
       </c>
@@ -15547,15 +15583,19 @@
       </c>
       <c r="E347" s="5" t="inlineStr">
         <is>
-          <t>التنفيذ</t>
+          <t>غير مصنف</t>
         </is>
       </c>
       <c r="F347" s="5" t="inlineStr">
         <is>
-          <t>إجرائي</t>
-        </is>
-      </c>
-      <c r="G347" s="5" t="inlineStr"/>
+          <t>قضائي تنظيمي</t>
+        </is>
+      </c>
+      <c r="G347" s="5" t="inlineStr">
+        <is>
+          <t>نظام القضاء ونظام ديوان المظالم</t>
+        </is>
+      </c>
       <c r="H347" s="5" t="n">
         <v>15</v>
       </c>
@@ -16058,7 +16098,7 @@
       </c>
       <c r="D359" s="5" t="inlineStr">
         <is>
-          <t>أخرى</t>
+          <t>تنظيم</t>
         </is>
       </c>
       <c r="E359" s="5" t="inlineStr">
@@ -18215,15 +18255,19 @@
       </c>
       <c r="E409" s="5" t="inlineStr">
         <is>
-          <t>التنفيذ</t>
+          <t>تنظيمي قطاعي</t>
         </is>
       </c>
       <c r="F409" s="5" t="inlineStr">
         <is>
-          <t>إجرائي</t>
-        </is>
-      </c>
-      <c r="G409" s="5" t="inlineStr"/>
+          <t>موضوعي/تنظيمي</t>
+        </is>
+      </c>
+      <c r="G409" s="5" t="inlineStr">
+        <is>
+          <t>نظام الأحداث</t>
+        </is>
+      </c>
       <c r="H409" s="5" t="n">
         <v>13</v>
       </c>
@@ -18731,15 +18775,19 @@
       </c>
       <c r="E421" s="5" t="inlineStr">
         <is>
-          <t>التنفيذ</t>
+          <t>الإداري والحوكمة العامة</t>
         </is>
       </c>
       <c r="F421" s="5" t="inlineStr">
         <is>
-          <t>إجرائي</t>
-        </is>
-      </c>
-      <c r="G421" s="5" t="inlineStr"/>
+          <t>موضوعي/تنظيمي</t>
+        </is>
+      </c>
+      <c r="G421" s="5" t="inlineStr">
+        <is>
+          <t>نظام المنافسات والمشتريات الحكومية</t>
+        </is>
+      </c>
       <c r="H421" s="5" t="n">
         <v>12</v>
       </c>
@@ -20322,15 +20370,19 @@
       </c>
       <c r="E458" s="5" t="inlineStr">
         <is>
-          <t>التنفيذ</t>
+          <t>الإداري والحوكمة العامة</t>
         </is>
       </c>
       <c r="F458" s="5" t="inlineStr">
         <is>
-          <t>إجرائي</t>
-        </is>
-      </c>
-      <c r="G458" s="5" t="inlineStr"/>
+          <t>موضوعي/تنظيمي</t>
+        </is>
+      </c>
+      <c r="G458" s="5" t="inlineStr">
+        <is>
+          <t>نظام المنافسات والمشتريات الحكومية</t>
+        </is>
+      </c>
       <c r="H458" s="5" t="n">
         <v>8</v>
       </c>
@@ -21571,7 +21623,7 @@
       </c>
       <c r="E487" s="2" t="inlineStr">
         <is>
-          <t>القضاء</t>
+          <t>التجاري والشركات</t>
         </is>
       </c>
       <c r="F487" s="2" t="inlineStr">
@@ -21630,7 +21682,7 @@
       </c>
       <c r="E488" s="2" t="inlineStr">
         <is>
-          <t>التوثيق والثروة العقارية</t>
+          <t>التوثيق</t>
         </is>
       </c>
       <c r="F488" s="2" t="inlineStr">
@@ -21689,12 +21741,12 @@
       </c>
       <c r="E489" s="2" t="inlineStr">
         <is>
-          <t>القضاء</t>
+          <t>الأحوال الشخصية</t>
         </is>
       </c>
       <c r="F489" s="2" t="inlineStr">
         <is>
-          <t>إجرائي</t>
+          <t>موضوعي/تنظيمي</t>
         </is>
       </c>
       <c r="G489" s="2" t="inlineStr">
@@ -21748,7 +21800,7 @@
       </c>
       <c r="E490" s="2" t="inlineStr">
         <is>
-          <t>القضاء</t>
+          <t>المرافعات والإجراءات</t>
         </is>
       </c>
       <c r="F490" s="2" t="inlineStr">
@@ -21807,7 +21859,7 @@
       </c>
       <c r="E491" s="2" t="inlineStr">
         <is>
-          <t>القضاء</t>
+          <t>المرافعات والإجراءات</t>
         </is>
       </c>
       <c r="F491" s="2" t="inlineStr">
@@ -21866,7 +21918,7 @@
       </c>
       <c r="E492" s="2" t="inlineStr">
         <is>
-          <t>القضاء</t>
+          <t>المرافعات والإجراءات</t>
         </is>
       </c>
       <c r="F492" s="2" t="inlineStr">
@@ -21925,7 +21977,7 @@
       </c>
       <c r="E493" s="2" t="inlineStr">
         <is>
-          <t>القضاء</t>
+          <t>المرافعات والإجراءات</t>
         </is>
       </c>
       <c r="F493" s="2" t="inlineStr">
@@ -21984,7 +22036,7 @@
       </c>
       <c r="E494" s="2" t="inlineStr">
         <is>
-          <t>القضاء</t>
+          <t>الإثبات</t>
         </is>
       </c>
       <c r="F494" s="2" t="inlineStr">
@@ -22043,7 +22095,7 @@
       </c>
       <c r="E495" s="2" t="inlineStr">
         <is>
-          <t>القضاء</t>
+          <t>الإثبات</t>
         </is>
       </c>
       <c r="F495" s="2" t="inlineStr">
@@ -22102,7 +22154,7 @@
       </c>
       <c r="E496" s="2" t="inlineStr">
         <is>
-          <t>القضاء</t>
+          <t>الإثبات</t>
         </is>
       </c>
       <c r="F496" s="2" t="inlineStr">
@@ -22159,10 +22211,14 @@
           <t>لائحة</t>
         </is>
       </c>
-      <c r="E497" s="2" t="inlineStr"/>
+      <c r="E497" s="2" t="inlineStr">
+        <is>
+          <t>الأحوال الشخصية</t>
+        </is>
+      </c>
       <c r="F497" s="2" t="inlineStr">
         <is>
-          <t>إجرائي</t>
+          <t>موضوعي/تنظيمي</t>
         </is>
       </c>
       <c r="G497" s="2" t="inlineStr">
@@ -22216,7 +22272,7 @@
       </c>
       <c r="E498" s="2" t="inlineStr">
         <is>
-          <t>المحاماة</t>
+          <t>المرافعات والإجراءات</t>
         </is>
       </c>
       <c r="F498" s="2" t="inlineStr">
@@ -22275,7 +22331,7 @@
       </c>
       <c r="E499" s="2" t="inlineStr">
         <is>
-          <t>القضاء</t>
+          <t>التجاري والشركات</t>
         </is>
       </c>
       <c r="F499" s="2" t="inlineStr">
@@ -22334,12 +22390,12 @@
       </c>
       <c r="E500" s="2" t="inlineStr">
         <is>
-          <t>الوثائق الأخرى</t>
+          <t>الشركات</t>
         </is>
       </c>
       <c r="F500" s="2" t="inlineStr">
         <is>
-          <t>إجرائي</t>
+          <t>موضوعي/تنظيمي</t>
         </is>
       </c>
       <c r="G500" s="2" t="inlineStr">
@@ -22391,10 +22447,14 @@
           <t>قواعد</t>
         </is>
       </c>
-      <c r="E501" s="2" t="inlineStr"/>
+      <c r="E501" s="2" t="inlineStr">
+        <is>
+          <t>الشركات</t>
+        </is>
+      </c>
       <c r="F501" s="2" t="inlineStr">
         <is>
-          <t>إجرائي</t>
+          <t>موضوعي/تنظيمي</t>
         </is>
       </c>
       <c r="G501" s="2" t="inlineStr">
@@ -23022,7 +23082,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>موضوعي/تنظيمي</t>
+          <t>إجرائي</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr"/>
@@ -23198,7 +23258,7 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>إجرائي</t>
+          <t>موضوعي/تنظيمي</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -23418,7 +23478,7 @@
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>إجرائي</t>
+          <t>موضوعي/تنظيمي</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -23456,7 +23516,7 @@
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>إجرائي</t>
+          <t>موضوعي/تنظيمي</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -23566,7 +23626,7 @@
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>إجرائي</t>
+          <t>موضوعي/تنظيمي</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -23600,7 +23660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -23652,79 +23712,101 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>الأنظمة الإجرائية</t>
+          <t>إجرائي</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>بتاريخ إصدار كامل موثّق — أنظمة أساسية</t>
+          <t>قضائي تنظيمي</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>بتاريخ إصدار كامل موثّق — لوائح وأدوات</t>
+          <t>بتاريخ إصدار كامل موثّق — أنظمة أساسية</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>بسنة إصدار من اسم النظام فقط</t>
+          <t>بتاريخ إصدار كامل موثّق — لوائح وأدوات</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>بلا تاريخ في القاعدة</t>
+          <t>بسنة إصدار من اسم النظام فقط</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>470</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>تاريخ التصدير</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
+          <t>بلا تاريخ في القاعدة</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>470</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
+          <t>تاريخ التصدير</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
           <t>ملاحظة</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>لم يُضَف أي تاريخ غير وارد في مصدر موثّق. تحويل الهجري للميلادي وفق تقويم أم القرى.</t>
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>ملاحظة</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>عمود «الطبيعة» تصنيف آلي بقواعد الاسم؛ واللوائح ترث مجال وطبيعة نظامها الأم.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B11"/>
+  <autoFilter ref="A1:B13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>